<commit_message>
Update to consider PoR case study
</commit_message>
<xml_diff>
--- a/inventories/lci-edm-i.xlsx
+++ b/inventories/lci-edm-i.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_transience\inventories\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_port_of_rotterdam\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459AAA29-2E5B-4FBB-AD9A-4C921316FBED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56ABC2BB-D555-4DFF-9BA0-60795C53C555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35535" yWindow="-18450" windowWidth="29040" windowHeight="17520" xr2:uid="{084DE41E-2059-4B64-8760-3FAEBCB66C1C}"/>
+    <workbookView xWindow="28740" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{084DE41E-2059-4B64-8760-3FAEBCB66C1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="203">
   <si>
     <t>database</t>
   </si>
@@ -462,9 +462,6 @@
     <t>market for argon, liquid</t>
   </si>
   <si>
-    <t>market for electric arc furnace converter</t>
-  </si>
-  <si>
     <t>market for electric arc furnace dust</t>
   </si>
   <si>
@@ -600,9 +597,6 @@
     <t>RU</t>
   </si>
   <si>
-    <t>Europe, without Russia and Türkiye</t>
-  </si>
-  <si>
     <t>RoE</t>
   </si>
   <si>
@@ -652,6 +646,9 @@
   </si>
   <si>
     <t>steel production, converter, low-alloyed, only primary steel</t>
+  </si>
+  <si>
+    <t>electric arc furnace construction</t>
   </si>
 </sst>
 </file>
@@ -729,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -751,7 +748,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -770,9 +766,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -810,7 +806,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -916,7 +912,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1058,7 +1054,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1071,6 +1067,7 @@
   <cols>
     <col min="1" max="1" width="50.3125" customWidth="1"/>
     <col min="2" max="2" width="12.41796875" customWidth="1"/>
+    <col min="3" max="3" width="35.47265625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.15625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1156,7 +1153,7 @@
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4134,13 +4131,13 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A172" t="s">
-        <v>140</v>
+        <v>202</v>
       </c>
       <c r="B172">
         <v>3.9999999999999998E-11</v>
       </c>
       <c r="C172" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D172" t="s">
         <v>9</v>
@@ -4151,7 +4148,7 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A173" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B173">
         <v>-1.9127399999999999E-2</v>
@@ -4168,7 +4165,7 @@
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A174" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B174">
         <v>-1.924E-2</v>
@@ -4185,7 +4182,7 @@
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A175" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B175">
         <v>-0.145866</v>
@@ -4202,13 +4199,13 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B176">
         <v>6.1701894910720287E-4</v>
       </c>
       <c r="C176" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D176" t="s">
         <v>35</v>
@@ -4219,13 +4216,13 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A177" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B177">
         <v>3.9197171088429527E-5</v>
       </c>
       <c r="C177" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D177" t="s">
         <v>35</v>
@@ -4236,13 +4233,13 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A178" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B178">
         <v>1.072302803147397E-2</v>
       </c>
       <c r="C178" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D178" t="s">
         <v>35</v>
@@ -4253,13 +4250,13 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B179">
         <v>9.0434291899349796E-3</v>
       </c>
       <c r="C179" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D179" t="s">
         <v>35</v>
@@ -4270,13 +4267,13 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A180" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B180">
         <v>4.9077363809222133E-2</v>
       </c>
       <c r="C180" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D180" t="s">
         <v>35</v>
@@ -4287,13 +4284,13 @@
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A181" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B181">
         <v>2.4149243635644229E-2</v>
       </c>
       <c r="C181" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D181" t="s">
         <v>35</v>
@@ -4304,13 +4301,13 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A182" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B182">
         <v>9.0621687446644332E-4</v>
       </c>
       <c r="C182" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D182" t="s">
         <v>35</v>
@@ -4321,13 +4318,13 @@
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A183" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B183">
         <v>1.750685094261555E-3</v>
       </c>
       <c r="C183" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D183" t="s">
         <v>35</v>
@@ -4338,13 +4335,13 @@
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A184" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B184">
         <v>6.3086297384941396E-3</v>
       </c>
       <c r="C184" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D184" t="s">
         <v>35</v>
@@ -4355,13 +4352,13 @@
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A185" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B185">
         <v>2.3658813269607248E-3</v>
       </c>
       <c r="C185" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D185" t="s">
         <v>35</v>
@@ -4372,13 +4369,13 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A186" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B186">
         <v>6.0557844051336374E-3</v>
       </c>
       <c r="C186" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D186" t="s">
         <v>35</v>
@@ -4389,13 +4386,13 @@
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A187" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B187">
         <v>4.2170956556704392E-4</v>
       </c>
       <c r="C187" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D187" t="s">
         <v>35</v>
@@ -4406,13 +4403,13 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A188" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B188">
         <v>1.3509107862769651E-3</v>
       </c>
       <c r="C188" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D188" t="s">
         <v>35</v>
@@ -4423,13 +4420,13 @@
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A189" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B189">
         <v>1.1264703406404729E-3</v>
       </c>
       <c r="C189" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D189" t="s">
         <v>35</v>
@@ -4440,13 +4437,13 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A190" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B190">
         <v>3.2423316654897009E-3</v>
       </c>
       <c r="C190" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D190" t="s">
         <v>35</v>
@@ -4457,13 +4454,13 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A191" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B191">
         <v>6.4981518778859382E-3</v>
       </c>
       <c r="C191" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D191" t="s">
         <v>35</v>
@@ -4474,13 +4471,13 @@
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A192" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B192">
         <v>4.7619389475090389E-2</v>
       </c>
       <c r="C192" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -4491,13 +4488,13 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A193" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B193">
         <v>1.362450118593771E-2</v>
       </c>
       <c r="C193" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D193" t="s">
         <v>35</v>
@@ -4508,13 +4505,13 @@
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A194" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B194">
         <v>1.5409829085202839E-2</v>
       </c>
       <c r="C194" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D194" t="s">
         <v>35</v>
@@ -4525,13 +4522,13 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A195" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B195">
         <v>2.1939409819286991E-3</v>
       </c>
       <c r="C195" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D195" t="s">
         <v>35</v>
@@ -4542,13 +4539,13 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A196" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B196">
         <v>8.2671317013689599E-3</v>
       </c>
       <c r="C196" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D196" t="s">
         <v>35</v>
@@ -4559,13 +4556,13 @@
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A197" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B197">
         <v>1.4478964264394961E-3</v>
       </c>
       <c r="C197" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D197" t="s">
         <v>35</v>
@@ -4576,13 +4573,13 @@
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A198" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B198">
         <v>1.396856486853193E-2</v>
       </c>
       <c r="C198" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D198" t="s">
         <v>35</v>
@@ -4593,13 +4590,13 @@
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A199" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B199">
         <v>4.7479539205062546E-3</v>
       </c>
       <c r="C199" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D199" t="s">
         <v>35</v>
@@ -4610,13 +4607,13 @@
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A200" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B200">
         <v>8.2127427674547768E-2</v>
       </c>
       <c r="C200" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D200" t="s">
         <v>35</v>
@@ -4627,13 +4624,13 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B201">
         <v>2.4472052767993819E-2</v>
       </c>
       <c r="C201" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D201" t="s">
         <v>35</v>
@@ -4644,13 +4641,13 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A202" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B202">
         <v>2.6205914037182531E-3</v>
       </c>
       <c r="C202" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D202" t="s">
         <v>35</v>
@@ -4661,13 +4658,13 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A203" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B203">
         <v>3.630578500388189E-3</v>
       </c>
       <c r="C203" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D203" t="s">
         <v>35</v>
@@ -4678,13 +4675,13 @@
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A204" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B204">
         <v>3.8909450495354721E-2</v>
       </c>
       <c r="C204" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D204" t="s">
         <v>35</v>
@@ -4695,13 +4692,13 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A205" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B205">
         <v>2.7850781556108671E-2</v>
       </c>
       <c r="C205" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D205" t="s">
         <v>35</v>
@@ -4712,13 +4709,13 @@
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A206" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B206">
         <v>9.0444166243619853E-3</v>
       </c>
       <c r="C206" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D206" t="s">
         <v>35</v>
@@ -4729,13 +4726,13 @@
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A207" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B207">
         <v>7.8782930409676283E-3</v>
       </c>
       <c r="C207" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D207" t="s">
         <v>35</v>
@@ -4746,13 +4743,13 @@
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A208" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B208">
         <v>6.1617203604531516E-3</v>
       </c>
       <c r="C208" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D208" t="s">
         <v>35</v>
@@ -4763,13 +4760,13 @@
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A209" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B209">
         <v>8.3223906299039627E-2</v>
       </c>
       <c r="C209" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D209" t="s">
         <v>35</v>
@@ -4780,13 +4777,13 @@
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A210" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B210">
         <v>1.439480743465304E-3</v>
       </c>
       <c r="C210" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D210" t="s">
         <v>35</v>
@@ -4797,13 +4794,13 @@
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A211" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B211">
         <v>5.4933228820234267E-3</v>
       </c>
       <c r="C211" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D211" t="s">
         <v>35</v>
@@ -4814,13 +4811,13 @@
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A212" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B212">
         <v>2.5084776215519189E-2</v>
       </c>
       <c r="C212" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D212" t="s">
         <v>35</v>
@@ -4831,13 +4828,13 @@
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B213">
         <v>8.2787002036942389E-4</v>
       </c>
       <c r="C213" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D213" t="s">
         <v>35</v>
@@ -4865,7 +4862,7 @@
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B215">
         <v>3.9169544357431502E-3</v>
@@ -4882,13 +4879,13 @@
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B216">
         <v>5.1107686432508084E-3</v>
       </c>
       <c r="C216" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D216" t="s">
         <v>10</v>
@@ -4899,13 +4896,13 @@
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B217">
         <v>4.0543827466608716E-3</v>
       </c>
       <c r="C217" t="s">
-        <v>186</v>
+        <v>26</v>
       </c>
       <c r="D217" t="s">
         <v>10</v>
@@ -4956,7 +4953,7 @@
         <v>4.3811603528579283E-5</v>
       </c>
       <c r="C220" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D220" t="s">
         <v>30</v>
@@ -4973,7 +4970,7 @@
         <v>1.8284972411520859E-4</v>
       </c>
       <c r="C221" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D221" t="s">
         <v>30</v>
@@ -4990,7 +4987,7 @@
         <v>7.8904791941083541E-5</v>
       </c>
       <c r="C222" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D222" t="s">
         <v>30</v>
@@ -5007,7 +5004,7 @@
         <v>3.4195994866009522E-4</v>
       </c>
       <c r="C223" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D223" t="s">
         <v>30</v>
@@ -5024,7 +5021,7 @@
         <v>1.1562776310568279E-3</v>
       </c>
       <c r="C224" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D224" t="s">
         <v>30</v>
@@ -5041,7 +5038,7 @@
         <v>3.5629885436650648E-4</v>
       </c>
       <c r="C225" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D225" t="s">
         <v>30</v>
@@ -5058,7 +5055,7 @@
         <v>1.164573403793201E-3</v>
       </c>
       <c r="C226" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D226" t="s">
         <v>30</v>
@@ -5075,7 +5072,7 @@
         <v>2.7926739785271148E-4</v>
       </c>
       <c r="C227" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D227" t="s">
         <v>30</v>
@@ -5092,7 +5089,7 @@
         <v>6.4076560632649634E-4</v>
       </c>
       <c r="C228" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D228" t="s">
         <v>30</v>
@@ -5109,7 +5106,7 @@
         <v>8.3557134767290182E-5</v>
       </c>
       <c r="C229" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D229" t="s">
         <v>30</v>
@@ -5126,7 +5123,7 @@
         <v>1.4560797988020699E-3</v>
       </c>
       <c r="C230" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D230" t="s">
         <v>30</v>
@@ -5143,7 +5140,7 @@
         <v>1.7040090788218631E-4</v>
       </c>
       <c r="C231" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D231" t="s">
         <v>30</v>
@@ -5160,7 +5157,7 @@
         <v>1.4314349753568329E-4</v>
       </c>
       <c r="C232" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D232" t="s">
         <v>30</v>
@@ -5177,7 +5174,7 @@
         <v>1.798089025848886E-5</v>
       </c>
       <c r="C233" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D233" t="s">
         <v>30</v>
@@ -5194,7 +5191,7 @@
         <v>9.7563381094070012E-5</v>
       </c>
       <c r="C234" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D234" t="s">
         <v>30</v>
@@ -5211,7 +5208,7 @@
         <v>8.2801613555683577E-5</v>
       </c>
       <c r="C235" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D235" t="s">
         <v>30</v>
@@ -5228,7 +5225,7 @@
         <v>5.1184918464480746E-4</v>
       </c>
       <c r="C236" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D236" t="s">
         <v>30</v>
@@ -5245,7 +5242,7 @@
         <v>3.9244120626921503E-5</v>
       </c>
       <c r="C237" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D237" t="s">
         <v>30</v>
@@ -5262,7 +5259,7 @@
         <v>6.3521910898943794E-4</v>
       </c>
       <c r="C238" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D238" t="s">
         <v>30</v>
@@ -5273,7 +5270,7 @@
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A239" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B239">
         <v>3.5972269319574498E-3</v>
@@ -5324,7 +5321,7 @@
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A242" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B242">
         <v>1.54919333848297E-2</v>
@@ -5341,7 +5338,7 @@
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A243" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B243">
         <v>3.6331804249169902E-7</v>
@@ -5358,7 +5355,7 @@
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A244" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B244">
         <v>1.21655250605964E-8</v>
@@ -5460,7 +5457,7 @@
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A250" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B250">
         <v>1.5491933384829701E-9</v>
@@ -5477,7 +5474,7 @@
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A251" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B251">
         <v>7.7008000000000005E-5</v>
@@ -5494,7 +5491,7 @@
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A252" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B252">
         <v>5.3103672189406999E-6</v>
@@ -5511,7 +5508,7 @@
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A253" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B253">
         <v>2.4494897427831801E-8</v>
@@ -5545,7 +5542,7 @@
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A255" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B255">
         <v>2E-8</v>
@@ -5562,7 +5559,7 @@
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A256" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B256">
         <v>7.7459666924148295E-8</v>
@@ -5630,7 +5627,7 @@
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B260">
         <v>5.1961524227066304E-6</v>
@@ -5647,7 +5644,7 @@
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A261" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B261">
         <v>1.4722431864335501E-5</v>
@@ -5664,7 +5661,7 @@
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B262">
         <v>2.2360679774997899E-10</v>
@@ -5681,7 +5678,7 @@
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B263">
         <v>3.2403703492039302E-5</v>
@@ -5715,7 +5712,7 @@
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B265">
         <v>2.19089023002066E-6</v>
@@ -5769,7 +5766,7 @@
         <v>1</v>
       </c>
       <c r="B269" s="14" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -5850,7 +5847,7 @@
     </row>
     <row r="278" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A278" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B278">
         <v>1</v>

</xml_diff>